<commit_message>
feat: add 3D tobacco warehouse digital twin web app for GitHub Pages
</commit_message>
<xml_diff>
--- a/Stock_Susunan_Bal_30_Agustus_2026.xlsx
+++ b/Stock_Susunan_Bal_30_Agustus_2026.xlsx
@@ -608,7 +608,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:T195"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -9688,7 +9688,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:H163"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -12688,7 +12688,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:T116"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.5" customWidth="1" min="1" max="1"/>
     <col width="9.5" customWidth="1" min="2" max="2"/>
@@ -18559,7 +18559,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:J391"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Update No Gudang Blok 01 Saf 4 ke 635 dan Blok 02 Saf 1 ke 634
</commit_message>
<xml_diff>
--- a/Stock_Susunan_Bal_30_Agustus_2026.xlsx
+++ b/Stock_Susunan_Bal_30_Agustus_2026.xlsx
@@ -977,16 +977,16 @@
         </is>
       </c>
       <c r="L11" s="11" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>35080</t>
+          <t>35663</t>
         </is>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>44 kg</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>35087</t>
+          <t>35080</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>45 kg</t>
         </is>
       </c>
       <c r="F22" s="11" t="n">
@@ -10713,7 +10713,7 @@
         <v>132</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>636</v>
@@ -10893,7 +10893,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>631</v>
@@ -13960,16 +13960,16 @@
         </is>
       </c>
       <c r="J7" s="18" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="K7" s="19" t="inlineStr">
         <is>
-          <t>35080</t>
+          <t>35663</t>
         </is>
       </c>
       <c r="L7" s="13" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>44 kg</t>
         </is>
       </c>
       <c r="M7" s="18" t="n">
@@ -14344,16 +14344,16 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>35087</t>
+          <t>35080</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>45 kg</t>
         </is>
       </c>
       <c r="D13" s="18" t="n">
@@ -20527,7 +20527,7 @@
         <v>6</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>1455</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -20557,7 +20557,7 @@
         <v>6</v>
       </c>
       <c r="I9" s="25" t="n">
-        <v>1448</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -21455,21 +21455,21 @@
         <v>10</v>
       </c>
       <c r="C38" s="31" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D38" s="32" t="inlineStr">
         <is>
-          <t>35080</t>
+          <t>35663</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F38" s="33" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>44 kg</t>
         </is>
       </c>
       <c r="G38" s="30" t="inlineStr">
@@ -22616,11 +22616,11 @@
         <v>37</v>
       </c>
       <c r="C65" s="18" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>35087</t>
+          <t>35080</t>
         </is>
       </c>
       <c r="E65" s="28" t="inlineStr">
@@ -22630,7 +22630,7 @@
       </c>
       <c r="F65" s="29" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>45 kg</t>
         </is>
       </c>
       <c r="G65" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Update Blok 7 Saf 2: ganti 697 menjadi 696
</commit_message>
<xml_diff>
--- a/Stock_Susunan_Bal_30_Agustus_2026.xlsx
+++ b/Stock_Susunan_Bal_30_Agustus_2026.xlsx
@@ -5159,16 +5159,16 @@
         </is>
       </c>
       <c r="F83" s="11" t="n">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="G83" s="12" t="inlineStr">
         <is>
-          <t>39096</t>
+          <t>39097</t>
         </is>
       </c>
       <c r="H83" s="13" t="inlineStr">
         <is>
-          <t>44 kg</t>
+          <t>39 kg</t>
         </is>
       </c>
       <c r="I83" s="11" t="n">
@@ -13043,7 +13043,7 @@
         <v>680</v>
       </c>
       <c r="D69" s="14" t="n">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E69" s="14" t="n">
         <v>693</v>
@@ -18206,16 +18206,16 @@
         </is>
       </c>
       <c r="D49" s="18" t="n">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E49" s="19" t="inlineStr">
         <is>
-          <t>39096</t>
+          <t>39097</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>44 kg</t>
+          <t>39 kg</t>
         </is>
       </c>
       <c r="G49" s="18" t="n">
@@ -23025,7 +23025,7 @@
         <v>7</v>
       </c>
       <c r="I14" s="23" t="n">
-        <v>1401</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -32932,11 +32932,11 @@
         <v>223</v>
       </c>
       <c r="C251" s="18" t="n">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="D251" s="19" t="inlineStr">
         <is>
-          <t>39096</t>
+          <t>39097</t>
         </is>
       </c>
       <c r="E251" s="28" t="inlineStr">
@@ -32946,7 +32946,7 @@
       </c>
       <c r="F251" s="29" t="inlineStr">
         <is>
-          <t>44 kg</t>
+          <t>39 kg</t>
         </is>
       </c>
       <c r="G251" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Tambahkan data pasangan bal ganti 930/961, 931/962, 963/242, 964/287 dan sinkronisasi laporan
</commit_message>
<xml_diff>
--- a/Stock_Susunan_Bal_30_Agustus_2026.xlsx
+++ b/Stock_Susunan_Bal_30_Agustus_2026.xlsx
@@ -2110,8 +2110,10 @@
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="11" t="inlineStr"/>
       <c r="K23" s="12" t="inlineStr"/>
-      <c r="L23" s="10" t="n">
-        <v>961</v>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>930/961</t>
+        </is>
       </c>
       <c r="M23" s="11" t="inlineStr">
         <is>
@@ -2120,11 +2122,13 @@
       </c>
       <c r="N23" s="12" t="inlineStr">
         <is>
-          <t>39.0 kg</t>
-        </is>
-      </c>
-      <c r="O23" s="10" t="n">
-        <v>962</v>
+          <t>39.0 kg/39.0 kg</t>
+        </is>
+      </c>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>931/962</t>
+        </is>
       </c>
       <c r="P23" s="11" t="inlineStr">
         <is>
@@ -2133,7 +2137,7 @@
       </c>
       <c r="Q23" s="12" t="inlineStr">
         <is>
-          <t>30.0 kg</t>
+          <t>30.0 kg/30.0 kg</t>
         </is>
       </c>
       <c r="R23" s="10" t="n">
@@ -3177,8 +3181,10 @@
       <c r="U36" s="10" t="inlineStr"/>
       <c r="V36" s="11" t="inlineStr"/>
       <c r="W36" s="12" t="inlineStr"/>
-      <c r="X36" s="10" t="n">
-        <v>964</v>
+      <c r="X36" s="10" t="inlineStr">
+        <is>
+          <t>964/287</t>
+        </is>
       </c>
       <c r="Y36" s="11" t="inlineStr">
         <is>
@@ -3190,8 +3196,10 @@
           <t>47.0 kg</t>
         </is>
       </c>
-      <c r="AA36" s="10" t="n">
-        <v>963</v>
+      <c r="AA36" s="10" t="inlineStr">
+        <is>
+          <t>963/242</t>
+        </is>
       </c>
       <c r="AB36" s="11" t="inlineStr">
         <is>
@@ -14236,11 +14244,15 @@
       <c r="C19" s="14" t="inlineStr"/>
       <c r="D19" s="14" t="inlineStr"/>
       <c r="E19" s="14" t="inlineStr"/>
-      <c r="F19" s="14" t="n">
-        <v>961</v>
-      </c>
-      <c r="G19" s="14" t="n">
-        <v>962</v>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>930/961</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>931/962</t>
+        </is>
       </c>
       <c r="H19" s="14" t="n">
         <v>960</v>
@@ -14545,11 +14557,15 @@
       <c r="G30" s="14" t="inlineStr"/>
       <c r="H30" s="14" t="inlineStr"/>
       <c r="I30" s="14" t="inlineStr"/>
-      <c r="J30" s="14" t="n">
-        <v>964</v>
-      </c>
-      <c r="K30" s="14" t="n">
-        <v>963</v>
+      <c r="J30" s="14" t="inlineStr">
+        <is>
+          <t>964/287</t>
+        </is>
+      </c>
+      <c r="K30" s="14" t="inlineStr">
+        <is>
+          <t>963/242</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -18735,8 +18751,10 @@
       <c r="G14" s="17" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="12" t="inlineStr"/>
-      <c r="J14" s="17" t="n">
-        <v>961</v>
+      <c r="J14" s="17" t="inlineStr">
+        <is>
+          <t>930/961</t>
+        </is>
       </c>
       <c r="K14" s="18" t="inlineStr">
         <is>
@@ -18745,11 +18763,13 @@
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>39.0 kg</t>
-        </is>
-      </c>
-      <c r="M14" s="17" t="n">
-        <v>962</v>
+          <t>39.0 kg/39.0 kg</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>931/962</t>
+        </is>
       </c>
       <c r="N14" s="18" t="inlineStr">
         <is>
@@ -18758,7 +18778,7 @@
       </c>
       <c r="O14" s="12" t="inlineStr">
         <is>
-          <t>30.0 kg</t>
+          <t>30.0 kg/30.0 kg</t>
         </is>
       </c>
       <c r="P14" s="17" t="n">
@@ -19522,8 +19542,10 @@
       <c r="S22" s="17" t="inlineStr"/>
       <c r="T22" s="18" t="inlineStr"/>
       <c r="U22" s="12" t="inlineStr"/>
-      <c r="V22" s="17" t="n">
-        <v>964</v>
+      <c r="V22" s="17" t="inlineStr">
+        <is>
+          <t>964/287</t>
+        </is>
       </c>
       <c r="W22" s="18" t="inlineStr">
         <is>
@@ -19535,8 +19557,10 @@
           <t>47.0 kg</t>
         </is>
       </c>
-      <c r="Y22" s="17" t="n">
-        <v>963</v>
+      <c r="Y22" s="17" t="inlineStr">
+        <is>
+          <t>963/242</t>
+        </is>
       </c>
       <c r="Z22" s="18" t="inlineStr">
         <is>
@@ -27469,7 +27493,7 @@
         <v>15</v>
       </c>
       <c r="I9" s="25" t="n">
-        <v>2298</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -27499,7 +27523,7 @@
         <v>21</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>2133</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -30774,8 +30798,10 @@
       <c r="B94" s="30" t="n">
         <v>66</v>
       </c>
-      <c r="C94" s="31" t="n">
-        <v>961</v>
+      <c r="C94" s="31" t="inlineStr">
+        <is>
+          <t>930/961</t>
+        </is>
       </c>
       <c r="D94" s="32" t="inlineStr">
         <is>
@@ -30784,12 +30810,12 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70/68</t>
         </is>
       </c>
       <c r="F94" s="33" t="inlineStr">
         <is>
-          <t>39.0 kg</t>
+          <t>39.0 kg/39.0 kg</t>
         </is>
       </c>
       <c r="G94" s="30" t="inlineStr">
@@ -30817,8 +30843,10 @@
       <c r="B95" s="28" t="n">
         <v>67</v>
       </c>
-      <c r="C95" s="17" t="n">
-        <v>962</v>
+      <c r="C95" s="17" t="inlineStr">
+        <is>
+          <t>931/962</t>
+        </is>
       </c>
       <c r="D95" s="18" t="inlineStr">
         <is>
@@ -30827,12 +30855,12 @@
       </c>
       <c r="E95" s="28" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70/68</t>
         </is>
       </c>
       <c r="F95" s="29" t="inlineStr">
         <is>
-          <t>30.0 kg</t>
+          <t>30.0 kg/30.0 kg</t>
         </is>
       </c>
       <c r="G95" s="28" t="inlineStr">
@@ -33096,8 +33124,10 @@
       <c r="B148" s="30" t="n">
         <v>120</v>
       </c>
-      <c r="C148" s="31" t="n">
-        <v>964</v>
+      <c r="C148" s="31" t="inlineStr">
+        <is>
+          <t>964/287</t>
+        </is>
       </c>
       <c r="D148" s="32" t="inlineStr">
         <is>
@@ -33139,8 +33169,10 @@
       <c r="B149" s="28" t="n">
         <v>121</v>
       </c>
-      <c r="C149" s="17" t="n">
-        <v>963</v>
+      <c r="C149" s="17" t="inlineStr">
+        <is>
+          <t>963/242</t>
+        </is>
       </c>
       <c r="D149" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sinkronisasi susunan bal dan pembersihan metadata master
</commit_message>
<xml_diff>
--- a/Stock_Susunan_Bal_30_Agustus_2026.xlsx
+++ b/Stock_Susunan_Bal_30_Agustus_2026.xlsx
@@ -2110,10 +2110,8 @@
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="11" t="inlineStr"/>
       <c r="K23" s="12" t="inlineStr"/>
-      <c r="L23" s="10" t="inlineStr">
-        <is>
-          <t>930/961</t>
-        </is>
+      <c r="L23" s="10" t="n">
+        <v>961</v>
       </c>
       <c r="M23" s="11" t="inlineStr">
         <is>
@@ -2122,13 +2120,11 @@
       </c>
       <c r="N23" s="12" t="inlineStr">
         <is>
-          <t>39.0 kg/39.0 kg</t>
-        </is>
-      </c>
-      <c r="O23" s="10" t="inlineStr">
-        <is>
-          <t>931/962</t>
-        </is>
+          <t>39.0 kg</t>
+        </is>
+      </c>
+      <c r="O23" s="10" t="n">
+        <v>962</v>
       </c>
       <c r="P23" s="11" t="inlineStr">
         <is>
@@ -2137,7 +2133,7 @@
       </c>
       <c r="Q23" s="12" t="inlineStr">
         <is>
-          <t>30.0 kg/30.0 kg</t>
+          <t>30.0 kg</t>
         </is>
       </c>
       <c r="R23" s="10" t="n">
@@ -3181,10 +3177,8 @@
       <c r="U36" s="10" t="inlineStr"/>
       <c r="V36" s="11" t="inlineStr"/>
       <c r="W36" s="12" t="inlineStr"/>
-      <c r="X36" s="10" t="inlineStr">
-        <is>
-          <t>964/287</t>
-        </is>
+      <c r="X36" s="10" t="n">
+        <v>964</v>
       </c>
       <c r="Y36" s="11" t="inlineStr">
         <is>
@@ -3196,10 +3190,8 @@
           <t>47.0 kg</t>
         </is>
       </c>
-      <c r="AA36" s="10" t="inlineStr">
-        <is>
-          <t>963/242</t>
-        </is>
+      <c r="AA36" s="10" t="n">
+        <v>963</v>
       </c>
       <c r="AB36" s="11" t="inlineStr">
         <is>
@@ -14244,15 +14236,11 @@
       <c r="C19" s="14" t="inlineStr"/>
       <c r="D19" s="14" t="inlineStr"/>
       <c r="E19" s="14" t="inlineStr"/>
-      <c r="F19" s="14" t="inlineStr">
-        <is>
-          <t>930/961</t>
-        </is>
-      </c>
-      <c r="G19" s="14" t="inlineStr">
-        <is>
-          <t>931/962</t>
-        </is>
+      <c r="F19" s="14" t="n">
+        <v>961</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>962</v>
       </c>
       <c r="H19" s="14" t="n">
         <v>960</v>
@@ -14557,15 +14545,11 @@
       <c r="G30" s="14" t="inlineStr"/>
       <c r="H30" s="14" t="inlineStr"/>
       <c r="I30" s="14" t="inlineStr"/>
-      <c r="J30" s="14" t="inlineStr">
-        <is>
-          <t>964/287</t>
-        </is>
-      </c>
-      <c r="K30" s="14" t="inlineStr">
-        <is>
-          <t>963/242</t>
-        </is>
+      <c r="J30" s="14" t="n">
+        <v>964</v>
+      </c>
+      <c r="K30" s="14" t="n">
+        <v>963</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
@@ -18751,10 +18735,8 @@
       <c r="G14" s="17" t="inlineStr"/>
       <c r="H14" s="18" t="inlineStr"/>
       <c r="I14" s="12" t="inlineStr"/>
-      <c r="J14" s="17" t="inlineStr">
-        <is>
-          <t>930/961</t>
-        </is>
+      <c r="J14" s="17" t="n">
+        <v>961</v>
       </c>
       <c r="K14" s="18" t="inlineStr">
         <is>
@@ -18763,13 +18745,11 @@
       </c>
       <c r="L14" s="12" t="inlineStr">
         <is>
-          <t>39.0 kg/39.0 kg</t>
-        </is>
-      </c>
-      <c r="M14" s="17" t="inlineStr">
-        <is>
-          <t>931/962</t>
-        </is>
+          <t>39.0 kg</t>
+        </is>
+      </c>
+      <c r="M14" s="17" t="n">
+        <v>962</v>
       </c>
       <c r="N14" s="18" t="inlineStr">
         <is>
@@ -18778,7 +18758,7 @@
       </c>
       <c r="O14" s="12" t="inlineStr">
         <is>
-          <t>30.0 kg/30.0 kg</t>
+          <t>30.0 kg</t>
         </is>
       </c>
       <c r="P14" s="17" t="n">
@@ -19542,10 +19522,8 @@
       <c r="S22" s="17" t="inlineStr"/>
       <c r="T22" s="18" t="inlineStr"/>
       <c r="U22" s="12" t="inlineStr"/>
-      <c r="V22" s="17" t="inlineStr">
-        <is>
-          <t>964/287</t>
-        </is>
+      <c r="V22" s="17" t="n">
+        <v>964</v>
       </c>
       <c r="W22" s="18" t="inlineStr">
         <is>
@@ -19557,10 +19535,8 @@
           <t>47.0 kg</t>
         </is>
       </c>
-      <c r="Y22" s="17" t="inlineStr">
-        <is>
-          <t>963/242</t>
-        </is>
+      <c r="Y22" s="17" t="n">
+        <v>963</v>
       </c>
       <c r="Z22" s="18" t="inlineStr">
         <is>
@@ -27493,7 +27469,7 @@
         <v>15</v>
       </c>
       <c r="I9" s="25" t="n">
-        <v>2229</v>
+        <v>2298</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -27523,7 +27499,7 @@
         <v>21</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>2037</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -30798,10 +30774,8 @@
       <c r="B94" s="30" t="n">
         <v>66</v>
       </c>
-      <c r="C94" s="31" t="inlineStr">
-        <is>
-          <t>930/961</t>
-        </is>
+      <c r="C94" s="31" t="n">
+        <v>961</v>
       </c>
       <c r="D94" s="32" t="inlineStr">
         <is>
@@ -30810,12 +30784,12 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>70/68</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F94" s="33" t="inlineStr">
         <is>
-          <t>39.0 kg/39.0 kg</t>
+          <t>39.0 kg</t>
         </is>
       </c>
       <c r="G94" s="30" t="inlineStr">
@@ -30843,10 +30817,8 @@
       <c r="B95" s="28" t="n">
         <v>67</v>
       </c>
-      <c r="C95" s="17" t="inlineStr">
-        <is>
-          <t>931/962</t>
-        </is>
+      <c r="C95" s="17" t="n">
+        <v>962</v>
       </c>
       <c r="D95" s="18" t="inlineStr">
         <is>
@@ -30855,12 +30827,12 @@
       </c>
       <c r="E95" s="28" t="inlineStr">
         <is>
-          <t>70/68</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F95" s="29" t="inlineStr">
         <is>
-          <t>30.0 kg/30.0 kg</t>
+          <t>30.0 kg</t>
         </is>
       </c>
       <c r="G95" s="28" t="inlineStr">
@@ -33124,10 +33096,8 @@
       <c r="B148" s="30" t="n">
         <v>120</v>
       </c>
-      <c r="C148" s="31" t="inlineStr">
-        <is>
-          <t>964/287</t>
-        </is>
+      <c r="C148" s="31" t="n">
+        <v>964</v>
       </c>
       <c r="D148" s="32" t="inlineStr">
         <is>
@@ -33169,10 +33139,8 @@
       <c r="B149" s="28" t="n">
         <v>121</v>
       </c>
-      <c r="C149" s="17" t="inlineStr">
-        <is>
-          <t>963/242</t>
-        </is>
+      <c r="C149" s="17" t="n">
+        <v>963</v>
       </c>
       <c r="D149" s="18" t="inlineStr">
         <is>

</xml_diff>